<commit_message>
Ajustes gerais / Publisher 3.0.0
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-BRIndividuoNaoIdentificado-1.0.xlsx
+++ b/output/StructureDefinition-BRIndividuoNaoIdentificado-1.0.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="153">
   <si>
     <t>Property</t>
   </si>
@@ -345,6 +345,12 @@
     <t>Sexo biológico obtido por meio de exame clínico ou de outros métodos diagnósticos referente ao indivíduo da hipótese de impossibilidade de identificação.</t>
   </si>
   <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>http://www.saude.gov.br/fhir/r4/ValueSet/BRSexo-1.0</t>
+  </si>
+  <si>
     <t>Extension.extension:gender.id</t>
   </si>
   <si>
@@ -456,6 +462,9 @@
   </si>
   <si>
     <t>Razão pela qual não foi possível obter os dados de identificação do indivíduo no contato assistencial.</t>
+  </si>
+  <si>
+    <t>http://www.saude.gov.br/fhir/r4/ValueSet/BRJustificativaIndividuoNaoIdentificado-1.0</t>
   </si>
   <si>
     <t>Extension.extension:reason.id</t>
@@ -849,7 +858,7 @@
     <col min="23" max="23" width="16.40625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="15.85546875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="18.19140625" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="16.2578125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="71.20703125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.2734375" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.1171875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.56640625" customWidth="true" bestFit="true"/>
@@ -1347,13 +1356,11 @@
         <v>81</v>
       </c>
       <c r="X5" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y5" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="Y5" s="2"/>
       <c r="Z5" t="s" s="2">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="AA5" t="s" s="2">
         <v>81</v>
@@ -1391,10 +1398,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1494,14 +1501,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" t="s" s="2">
@@ -1523,13 +1530,13 @@
         <v>98</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="N7" t="s" s="2">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
@@ -1599,10 +1606,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1625,16 +1632,16 @@
         <v>81</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1684,7 +1691,7 @@
         <v>81</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>83</v>
@@ -1699,15 +1706,15 @@
         <v>81</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1730,13 +1737,13 @@
         <v>81</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1787,7 +1794,7 @@
         <v>81</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>82</v>
@@ -1799,21 +1806,21 @@
         <v>81</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B10" t="s" s="2">
         <v>96</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>81</v>
@@ -1838,10 +1845,10 @@
         <v>98</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1912,10 +1919,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2015,14 +2022,14 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
@@ -2044,13 +2051,13 @@
         <v>98</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="N12" t="s" s="2">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
@@ -2120,10 +2127,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2146,16 +2153,16 @@
         <v>81</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2163,7 +2170,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>81</v>
@@ -2205,7 +2212,7 @@
         <v>81</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>83</v>
@@ -2220,15 +2227,15 @@
         <v>81</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2251,13 +2258,13 @@
         <v>81</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2308,7 +2315,7 @@
         <v>81</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>82</v>
@@ -2320,21 +2327,21 @@
         <v>81</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>96</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>81</v>
@@ -2359,10 +2366,10 @@
         <v>98</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2389,13 +2396,11 @@
         <v>81</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y15" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="Y15" s="2"/>
       <c r="Z15" t="s" s="2">
-        <v>81</v>
+        <v>146</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>81</v>
@@ -2433,10 +2438,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2536,14 +2541,14 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
@@ -2565,13 +2570,13 @@
         <v>98</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -2641,10 +2646,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2667,16 +2672,16 @@
         <v>81</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2684,7 +2689,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>81</v>
@@ -2726,7 +2731,7 @@
         <v>81</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>83</v>
@@ -2741,15 +2746,15 @@
         <v>81</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2772,13 +2777,13 @@
         <v>81</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2829,7 +2834,7 @@
         <v>81</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>82</v>
@@ -2841,18 +2846,18 @@
         <v>81</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2875,16 +2880,16 @@
         <v>81</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -2934,7 +2939,7 @@
         <v>81</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>83</v>
@@ -2949,15 +2954,15 @@
         <v>81</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2980,13 +2985,13 @@
         <v>81</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3037,7 +3042,7 @@
         <v>81</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>82</v>
@@ -3049,10 +3054,10 @@
         <v>81</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>